<commit_message>
feat(trips): isolate soft deleted trip ref_ids to TRP-DEL- prefix and handle gapless restoration
</commit_message>
<xml_diff>
--- a/Trucks Docs (1)/Trucks Docs/mandatory_documents_audit_single_sheet.xlsx
+++ b/Trucks Docs (1)/Trucks Docs/mandatory_documents_audit_single_sheet.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,8 +66,14 @@
       <color rgb="009F1239"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00854D0E"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -104,6 +110,12 @@
         <bgColor rgb="00FECDD3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF9C3"/>
+        <bgColor rgb="00FEF9C3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -131,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -153,6 +165,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -521,38 +536,38 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MERCON LOGISTICS - VEHICLE COMPLIANCE AUDIT (100% MATCH WITH FRONTEND UI)</t>
+          <t>MERCON FLEET - MANDATORY DOCUMENTS AUDIT (MISSING &amp; EXPIRY REPORT)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Audit Date: August 26, 2026 | Fleet Size: 31 Trucks | Verified 1-to-1 against Live System UI Dashboard Cards</t>
+          <t>Audit Date: August 26, 2026 | Total Fleet: 31 Trucks | Mandatory Required Docs: Istimara, Insurance, Operation Card, FAHAS, SASO/UPD</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Fleet Summary: 31 Trucks Total | 24 Trucks Need Action (17 Missing Docs, 27 Expired Docs) | 7 Compliant Trucks</t>
+          <t>Fleet Summary: 31 Trucks Total | 27 Need Action (20 Missing, 20 Expired)</t>
         </is>
       </c>
     </row>
@@ -604,19 +619,19 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>UI Action Status</t>
+          <t>Action Status</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>TRK-127</t>
+          <t>TRK-115</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>KSA-6102</t>
+          <t>ESA-4207</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -629,14 +644,14 @@
           <t>MISSING</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -645,62 +660,62 @@
         </is>
       </c>
       <c r="H7" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I7" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>🚨 3 Issues</t>
+          <t>ACTION NEEDED (5 Issues)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>TRK-115</t>
+          <t>TRK-127</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>ESA-4207</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-02-17)</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
+          <t>KSA-6102</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2026-12-17)</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2026-12-27)</t>
+        </is>
+      </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="H8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="I8" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>🚨 3 Issues</t>
+          <t>ACTION NEEDED (3 Issues)</t>
         </is>
       </c>
     </row>
@@ -717,12 +732,12 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-02-21)</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -748,178 +763,178 @@
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>🚨 3 Issues</t>
+          <t>ACTION NEEDED (3 Issues)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>TRK-110</t>
+          <t>TRK-131</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>VRA-5510</t>
+          <t>DRA-6487</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-02-23)</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-02-17)</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2027-06-17)</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Expiring in 67d (2026-11-01)</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>EXPIRED (2025-09-21)</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="n">
-        <v>0</v>
+          <t>EXPIRED (2026-08-21)</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>🚨 3 Issues</t>
+          <t>ACTION NEEDED (3 Issues)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>TRK-114</t>
+          <t>TRK-112</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>ESA-4244</t>
+          <t>BRA-5309</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-06-19)</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="n">
+          <t>VALID (2027-04-11)</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>EXPIRED (2025-07-20)</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Expiring in 81d (2026-11-15)</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I11" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>🚨 2 Issues</t>
+          <t>ACTION NEEDED (3 Issues)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>TRK-116</t>
+          <t>TRK-122</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>ZSA-5049</t>
+          <t>DRA-6485</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-06-19)</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="n">
+          <t>VALID (2027-04-13)</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-05-01)</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Expiring in 56d (2026-10-21)</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I12" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>🚨 2 Issues</t>
+          <t>ACTION NEEDED (3 Issues)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>TRK-121</t>
+          <t>TRK-114</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>DRA-6455</t>
+          <t>ESA-4244</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-06-19)</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2027-02-21)</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-01-02)</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -927,52 +942,52 @@
           <t>MISSING</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="H13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>🚨 2 Issues</t>
+          <t>ACTION NEEDED (2 Issues)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>TRK-131</t>
+          <t>TRK-116</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>DRA-6487</t>
+          <t>ZSA-5049</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-02-21)</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-08-21)</t>
+          <t>VALID (2027-04-11)</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -981,41 +996,41 @@
         </is>
       </c>
       <c r="H14" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I14" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>🚨 2 Issues</t>
+          <t>ACTION NEEDED (2 Issues)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>TRK-123</t>
+          <t>TRK-121</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>USA-6010</t>
+          <t>DRA-6455</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-08-03)</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-06-19)</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2027-04-14)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1025,7 +1040,7 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2026-12-03)</t>
         </is>
       </c>
       <c r="H15" s="6" t="n">
@@ -1036,72 +1051,72 @@
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>🚨 2 Issues</t>
+          <t>ACTION NEEDED (2 Issues)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>TRK-117</t>
+          <t>TRK-123</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>BRA-4012</t>
+          <t>USA-6010</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-06-19)</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-07-21)</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2027-02-21)</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-08-03)</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="H16" s="7" t="n">
-        <v>0</v>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>🚨 2 Issues</t>
+          <t>ACTION NEEDED (2 Issues)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>TRK-112</t>
+          <t>TRK-117</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>BRA-5309</t>
+          <t>BRA-4012</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -1111,17 +1126,17 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-04-11)</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>EXPIRED (2025-07-20)</t>
+          <t>EXPIRED (2026-07-21)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -1132,24 +1147,24 @@
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>🚨 2 Issues</t>
+          <t>ACTION NEEDED (2 Issues)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>TRK-122</t>
+          <t>TRK-113</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>DRA-6485</t>
+          <t>VRA-3358</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -1159,17 +1174,17 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-04-11)</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-05-01)</t>
+          <t>EXPIRED (2026-07-14)</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -1180,44 +1195,44 @@
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>🚨 2 Issues</t>
+          <t>ACTION NEEDED (2 Issues)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>TRK-103</t>
+          <t>TRK-110</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>SRA-6706</t>
+          <t>VRA-5510</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-02-23)</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2027-02-21)</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-02-17)</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-07-21)</t>
+          <t>EXPIRED (2025-09-21)</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -1228,168 +1243,168 @@
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>🚨 2 Issues</t>
+          <t>ACTION NEEDED (2 Issues)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>TRK-104</t>
+          <t>TRK-118</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>SRA-6708</t>
+          <t>LSA-3999</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-02-23)</t>
+          <t>EXPIRED (2026-06-19)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2025-07-20)</t>
+          <t>VALID (2027-04-11)</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Expiring in 43d (2026-10-08)</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>🚨 2 Issues</t>
+          <t>ACTION NEEDED (2 Issues)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>TRK-101</t>
+          <t>TRK-109</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>UDA-2541</t>
+          <t>ERA-3531</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-02-23)</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-02-17)</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2027-02-21)</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2027-02-19)</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Expiring in 90d (2026-11-24)</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>Expiring in 59d (2026-10-24)</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="8" t="n">
-        <v>2</v>
+      <c r="I21" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>🚨 2 Issues</t>
+          <t>ACTION NEEDED (2 Issues)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>TRK-113</t>
+          <t>TRK-129</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>VRA-3358</t>
+          <t>DRA-6484</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-06-19)</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-07-14)</t>
+          <t>VALID (2027-04-11)</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2026-12-25)</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="H22" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="8" t="n">
-        <v>2</v>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>🚨 2 Issues</t>
+          <t>ACTION NEEDED (1 Issues)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>TRK-129</t>
+          <t>TRK-128</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>DRA-6484</t>
+          <t>NXA-8210</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1399,17 +1414,17 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-06-11)</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-05-19)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H23" s="6" t="n">
@@ -1420,24 +1435,24 @@
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>🚨 1 Issues</t>
+          <t>ACTION NEEDED (1 Issues)</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>TRK-128</t>
+          <t>TRK-119</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>NXA-8210</t>
+          <t>VTA-3241</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1447,17 +1462,17 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-06-11)</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-05-19)</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H24" s="6" t="n">
@@ -1468,44 +1483,44 @@
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>🚨 1 Issues</t>
+          <t>ACTION NEEDED (1 Issues)</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>TRK-119</t>
+          <t>TRK-108</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>VTA-3241</t>
+          <t>XXA-4293</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2027-05-16)</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
-        </is>
-      </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H25" s="6" t="n">
@@ -1516,92 +1531,92 @@
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>🚨 1 Issues</t>
+          <t>ACTION NEEDED (1 Issues)</t>
         </is>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>TRK-108</t>
+          <t>TRK-103</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>XXA-4293</t>
+          <t>SRA-6706</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-02-21)</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>VALID (2027-04-11)</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-07-21)</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="n">
+          <t>VALID (2026-12-02)</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="I26" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>🚨 1 Issues</t>
+          <t>ACTION NEEDED (1 Issues)</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>TRK-107</t>
+          <t>TRK-104</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>EXA-5999</t>
+          <t>SRA-6708</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-02-21)</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-02-19)</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-01-15)</t>
+          <t>EXPIRED (2025-07-20)</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -1612,44 +1627,44 @@
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>🚨 1 Issues</t>
+          <t>ACTION NEEDED (1 Issues)</t>
         </is>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>TRK-118</t>
+          <t>TRK-101</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>LSA-3999</t>
+          <t>UDA-2541</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-06-19)</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2027-02-21)</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-02-17)</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-03-18)</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -1660,44 +1675,44 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>🚨 1 Issues</t>
+          <t>ACTION NEEDED (1 Issues)</t>
         </is>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>TRK-124</t>
+          <t>TRK-106</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>TRA-9153</t>
+          <t>VSA-3071</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-06-19)</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2027-02-21)</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
+          <t>VALID (2027-02-19)</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-04-20)</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -1708,92 +1723,92 @@
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>🚨 1 Issues</t>
+          <t>ACTION NEEDED (1 Issues)</t>
         </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>TRK-106</t>
+          <t>TRK-130</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>VSA-3071</t>
+          <t>DRA-6456</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-04-20)</t>
+          <t>VALID (2027-06-17)</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Expiring in 67d (2026-11-01)</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>VALID (2027-07-29)</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I30" s="8" t="n">
-        <v>1</v>
+      <c r="I30" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>🚨 1 Issues</t>
+          <t>ACTION NEEDED (1 Issues)</t>
         </is>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>TRK-130</t>
+          <t>TRK-102</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>DRA-6456</t>
+          <t>DRA-9973</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-02-21)</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-02-19)</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
+          <t>VALID (2026-11-25)</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>Expiring in 59d (2026-10-24)</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -1802,46 +1817,46 @@
       <c r="I31" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>✔ Compliant</t>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>ACTION NEEDED (1 Issues)</t>
         </is>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>TRK-102</t>
+          <t>TRK-126</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>DRA-9973</t>
+          <t>KSA-6097</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Expiring in 72d (2026-11-06)</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2026-12-17)</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -1850,46 +1865,46 @@
       <c r="I32" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J32" s="7" t="inlineStr">
-        <is>
-          <t>✔ Compliant</t>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>ACTION NEEDED (1 Issues)</t>
         </is>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>TRK-109</t>
+          <t>TRK-125</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>ERA-3531</t>
+          <t>KSA-6098</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>Expiring in 72d (2026-11-06)</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2026-12-17)</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2026-12-02)</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -1898,9 +1913,9 @@
       <c r="I33" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="7" t="inlineStr">
-        <is>
-          <t>✔ Compliant</t>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>ACTION NEEDED (1 Issues)</t>
         </is>
       </c>
     </row>
@@ -1917,27 +1932,27 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-06-04)</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-06-06)</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-04-13)</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-04-12)</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -1948,44 +1963,44 @@
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>✔ Compliant</t>
+          <t>OK (Compliant)</t>
         </is>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>TRK-126</t>
+          <t>TRK-107</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>KSA-6097</t>
+          <t>EXA-5999</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-02-12)</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2026-12-18)</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-01-25)</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -1996,44 +2011,44 @@
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>✔ Compliant</t>
+          <t>OK (Compliant)</t>
         </is>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>TRK-125</t>
+          <t>TRK-105</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>KSA-6098</t>
+          <t>NDA-5085</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-02-21)</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-02-19)</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-01-25)</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -2044,44 +2059,44 @@
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>✔ Compliant</t>
+          <t>OK (Compliant)</t>
         </is>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>TRK-105</t>
+          <t>TRK-124</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>NDA-5085</t>
+          <t>TRA-9153</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (No Expiry Date)</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-06-17)</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2027-04-11)</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2026-12-31)</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>VALID (2026-12-02)</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -2092,14 +2107,14 @@
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>✔ Compliant</t>
+          <t>OK (Compliant)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A4:B4"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A4:J4"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>